<commit_message>
Update of the Documents
</commit_message>
<xml_diff>
--- a/S2_Planning_projet.xlsx
+++ b/S2_Planning_projet.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\event\Desktop\Projet\Bachelor 2026-2027\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F31C9FE5-C3C3-4AA8-AE45-99FA9D360CF7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8264840C-390A-438D-BE36-743E0E466E11}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" tabRatio="500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Mode d'emploi" sheetId="1" r:id="rId1"/>
@@ -44,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="233" uniqueCount="206">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="238" uniqueCount="210">
   <si>
     <t>Séance 2 · un seul classeur par équipe, déposé dans l'espace partagé</t>
   </si>
@@ -628,9 +628,6 @@
     <t>Chef du Projet</t>
   </si>
   <si>
-    <t>Dimytro DUDAR</t>
-  </si>
-  <si>
     <t>Referent Technique</t>
   </si>
   <si>
@@ -662,6 +659,21 @@
   </si>
   <si>
     <t>R</t>
+  </si>
+  <si>
+    <t>Oui</t>
+  </si>
+  <si>
+    <t>25/11/2026</t>
+  </si>
+  <si>
+    <t>21/10/2026</t>
+  </si>
+  <si>
+    <t>dmdu1014@eleve.isep.fr</t>
+  </si>
+  <si>
+    <t>Dymitro DUDAR</t>
   </si>
 </sst>
 </file>
@@ -952,20 +964,20 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="2" xfId="2" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1004,7 +1016,7 @@
     <xf numFmtId="0" fontId="9" fillId="6" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="7" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="2" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -1411,18 +1423,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="30" t="s">
+      <c r="A1" s="31" t="s">
         <v>190</v>
       </c>
-      <c r="B1" s="30"/>
-      <c r="C1" s="30"/>
+      <c r="B1" s="31"/>
+      <c r="C1" s="31"/>
     </row>
     <row r="2" spans="1:3" ht="30" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="32" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="31"/>
-      <c r="C2" s="31"/>
+      <c r="B2" s="32"/>
+      <c r="C2" s="32"/>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.3">
       <c r="A3" s="4"/>
@@ -1433,86 +1445,86 @@
       <c r="A4" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="32" t="s">
+      <c r="B4" s="30" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="32"/>
+      <c r="C4" s="30"/>
     </row>
     <row r="5" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="32" t="s">
+      <c r="B5" s="30" t="s">
         <v>4</v>
       </c>
-      <c r="C5" s="32"/>
+      <c r="C5" s="30"/>
     </row>
     <row r="6" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="B6" s="32" t="s">
+      <c r="B6" s="30" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="32"/>
+      <c r="C6" s="30"/>
     </row>
     <row r="7" spans="1:3" ht="56.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="B7" s="32" t="s">
+      <c r="B7" s="30" t="s">
         <v>8</v>
       </c>
-      <c r="C7" s="32"/>
+      <c r="C7" s="30"/>
     </row>
     <row r="8" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="B8" s="32" t="s">
+      <c r="B8" s="30" t="s">
         <v>10</v>
       </c>
-      <c r="C8" s="32"/>
+      <c r="C8" s="30"/>
     </row>
     <row r="9" spans="1:3" ht="69.599999999999994" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="B9" s="32" t="s">
+      <c r="B9" s="30" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="32"/>
+      <c r="C9" s="30"/>
     </row>
     <row r="10" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="32" t="s">
+      <c r="B10" s="30" t="s">
         <v>14</v>
       </c>
-      <c r="C10" s="32"/>
+      <c r="C10" s="30"/>
     </row>
     <row r="11" spans="1:3" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="B11" s="32" t="s">
+      <c r="B11" s="30" t="s">
         <v>16</v>
       </c>
-      <c r="C11" s="32"/>
+      <c r="C11" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="10">
+    <mergeCell ref="A1:C1"/>
+    <mergeCell ref="A2:C2"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="B5:C5"/>
+    <mergeCell ref="B6:C6"/>
     <mergeCell ref="B7:C7"/>
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="B9:C9"/>
     <mergeCell ref="B10:C10"/>
     <mergeCell ref="B11:C11"/>
-    <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A2:C2"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="B5:C5"/>
-    <mergeCell ref="B6:C6"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -1945,10 +1957,10 @@
         <v>193</v>
       </c>
       <c r="C5" s="10" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="D5" s="27" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="E5" s="14">
         <v>36</v>
@@ -1964,15 +1976,17 @@
     </row>
     <row r="6" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="10" t="s">
+        <v>209</v>
+      </c>
+      <c r="B6" s="10" t="s">
         <v>194</v>
       </c>
-      <c r="B6" s="10" t="s">
-        <v>195</v>
-      </c>
       <c r="C6" s="10" t="s">
-        <v>197</v>
-      </c>
-      <c r="D6" s="10"/>
+        <v>196</v>
+      </c>
+      <c r="D6" s="27" t="s">
+        <v>208</v>
+      </c>
       <c r="E6" s="14">
         <v>36</v>
       </c>
@@ -1987,16 +2001,16 @@
     </row>
     <row r="7" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="10" t="s">
+        <v>195</v>
+      </c>
+      <c r="B7" s="10" t="s">
         <v>196</v>
       </c>
-      <c r="B7" s="10" t="s">
-        <v>197</v>
-      </c>
       <c r="C7" s="10" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="D7" s="27" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="E7" s="14">
         <v>36</v>
@@ -2041,7 +2055,7 @@
         <v>62</v>
       </c>
       <c r="B10" s="39" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C10" s="40"/>
       <c r="D10" s="40"/>
@@ -2054,7 +2068,7 @@
         <v>63</v>
       </c>
       <c r="B11" s="39" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C11" s="40"/>
       <c r="D11" s="40"/>
@@ -2090,6 +2104,7 @@
     <hyperlink ref="B10" r:id="rId2" xr:uid="{13B79908-F992-4A66-8A87-5ECFC2156B7C}"/>
     <hyperlink ref="B11" r:id="rId3" xr:uid="{C772EF2E-CEB3-4087-877D-6D1DB24417F0}"/>
     <hyperlink ref="D7" r:id="rId4" xr:uid="{F671C662-2025-4DC2-93C6-893365602FEE}"/>
+    <hyperlink ref="D6" r:id="rId5" xr:uid="{290CB932-CA29-42F2-AB5F-C836308D12BE}"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.5"/>
   <pageSetup fitToHeight="0" orientation="landscape" horizontalDpi="300" verticalDpi="300"/>
@@ -2112,12 +2127,12 @@
     <col min="3" max="3" width="38" customWidth="1"/>
     <col min="4" max="4" width="32" customWidth="1"/>
     <col min="5" max="5" width="18" customWidth="1"/>
-    <col min="6" max="6" width="9" customWidth="1"/>
+    <col min="6" max="6" width="12.33203125" customWidth="1"/>
     <col min="7" max="7" width="13.6640625" customWidth="1"/>
     <col min="8" max="8" width="18.44140625" customWidth="1"/>
     <col min="9" max="9" width="15.109375" customWidth="1"/>
     <col min="10" max="11" width="8" customWidth="1"/>
-    <col min="12" max="12" width="12" customWidth="1"/>
+    <col min="12" max="12" width="15.21875" customWidth="1"/>
     <col min="13" max="13" width="11" customWidth="1"/>
     <col min="14" max="14" width="26" customWidth="1"/>
   </cols>
@@ -2275,7 +2290,7 @@
         <v>86</v>
       </c>
       <c r="E6" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F6" s="18">
         <v>2</v>
@@ -2316,7 +2331,7 @@
         <v>89</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>194</v>
+        <v>209</v>
       </c>
       <c r="F7" s="18">
         <v>2</v>
@@ -2400,7 +2415,7 @@
         <v>95</v>
       </c>
       <c r="E9" s="18" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="F9" s="18">
         <v>2</v>
@@ -3869,9 +3884,8 @@
         <f>IF(Tâches!$C7="","",Tâches!$C7)</f>
         <v>Relever le matériel de l'équipe</v>
       </c>
-      <c r="C8" s="14" t="str">
-        <f>IF(Tâches!$C7="","",Tâches!$E7&amp;"")</f>
-        <v>Dimytro DUDAR</v>
+      <c r="C8" s="14" t="s">
+        <v>209</v>
       </c>
       <c r="D8" s="14" t="str">
         <f>IF(Tâches!$C7="","",Tâches!$M7&amp;"")</f>
@@ -7332,7 +7346,9 @@
       <c r="E5" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="F5" s="14"/>
+      <c r="F5" s="14" t="s">
+        <v>205</v>
+      </c>
       <c r="G5" s="26">
         <v>46309</v>
       </c>
@@ -7347,7 +7363,9 @@
       <c r="C6" s="14" t="s">
         <v>122</v>
       </c>
-      <c r="D6" s="26"/>
+      <c r="D6" s="26" t="s">
+        <v>207</v>
+      </c>
       <c r="E6" s="10" t="s">
         <v>123</v>
       </c>
@@ -7364,7 +7382,9 @@
       <c r="C7" s="14" t="s">
         <v>126</v>
       </c>
-      <c r="D7" s="26"/>
+      <c r="D7" s="26" t="s">
+        <v>206</v>
+      </c>
       <c r="E7" s="10" t="s">
         <v>127</v>
       </c>
@@ -7381,7 +7401,9 @@
       <c r="C8" s="14" t="s">
         <v>130</v>
       </c>
-      <c r="D8" s="26"/>
+      <c r="D8" s="26">
+        <v>46065</v>
+      </c>
       <c r="E8" s="10" t="s">
         <v>131</v>
       </c>
@@ -7398,7 +7420,9 @@
       <c r="C9" s="14" t="s">
         <v>134</v>
       </c>
-      <c r="D9" s="26"/>
+      <c r="D9" s="26">
+        <v>46277</v>
+      </c>
       <c r="E9" s="10" t="s">
         <v>135</v>
       </c>
@@ -7446,15 +7470,15 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+      <c r="A1" s="28" t="s">
         <v>136</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-      <c r="F1" s="46"/>
-      <c r="G1" s="46"/>
+      <c r="B1" s="28"/>
+      <c r="C1" s="28"/>
+      <c r="D1" s="28"/>
+      <c r="E1" s="28"/>
+      <c r="F1" s="28"/>
+      <c r="G1" s="28"/>
     </row>
     <row r="2" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">
@@ -7489,7 +7513,7 @@
       </c>
       <c r="D4" s="14" t="str">
         <f>IF(Équipe!A6="","Membre 2",Équipe!A6)</f>
-        <v>Dimytro DUDAR</v>
+        <v>Dymitro DUDAR</v>
       </c>
       <c r="E4" s="14" t="str">
         <f>IF(Équipe!A7="","Membre 3",Équipe!A7)</f>
@@ -7511,7 +7535,7 @@
         <v>141</v>
       </c>
       <c r="C5" s="14" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D5" s="14"/>
       <c r="E5" s="14"/>
@@ -7529,13 +7553,13 @@
         <v>143</v>
       </c>
       <c r="C6" s="14" t="s">
+        <v>203</v>
+      </c>
+      <c r="D6" s="14" t="s">
         <v>204</v>
       </c>
-      <c r="D6" s="14" t="s">
-        <v>205</v>
-      </c>
       <c r="E6" s="14" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F6" s="14"/>
       <c r="G6" s="14" t="str">
@@ -7789,21 +7813,21 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="27.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="28" t="s">
+      <c r="A1" s="46" t="s">
         <v>157</v>
       </c>
-      <c r="B1" s="28"/>
-      <c r="C1" s="28"/>
-      <c r="D1" s="28"/>
-      <c r="E1" s="28"/>
-      <c r="F1" s="28"/>
-      <c r="G1" s="28"/>
-      <c r="H1" s="28"/>
-      <c r="I1" s="28"/>
-      <c r="J1" s="28"/>
-      <c r="K1" s="28"/>
-      <c r="L1" s="28"/>
-      <c r="M1" s="28"/>
+      <c r="B1" s="46"/>
+      <c r="C1" s="46"/>
+      <c r="D1" s="46"/>
+      <c r="E1" s="46"/>
+      <c r="F1" s="46"/>
+      <c r="G1" s="46"/>
+      <c r="H1" s="46"/>
+      <c r="I1" s="46"/>
+      <c r="J1" s="46"/>
+      <c r="K1" s="46"/>
+      <c r="L1" s="46"/>
+      <c r="M1" s="46"/>
     </row>
     <row r="2" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="29" t="s">

</xml_diff>